<commit_message>
Sprint 3 final acceptance test
</commit_message>
<xml_diff>
--- a/etc/Updated Acceptance Test plan.xlsx
+++ b/etc/Updated Acceptance Test plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="176">
   <si>
     <t>Instructions</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>HS; 7/7</t>
+  </si>
+  <si>
+    <t>HS; 7/27;</t>
   </si>
   <si>
     <t>Given I am a new user, when I try to make an account with a taken username, the system refuses the attempt and offers to redirect to login.</t>
@@ -326,6 +329,249 @@
     <t>HS; 7/7; basket is not saved in account information, there is a singlular shared basked that shows up for everything
 UPDATE: each helper has a seperate basket that loads, now passes</t>
   </si>
+  <si>
+    <t>As a user, I want to view all organizations in the system so I know which ones are present.</t>
+  </si>
+  <si>
+    <t>Given I have a valid account, when I am logged in, I can see a link to the organizations view in the navbar</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my account, when I navigate to the organizations view, I can see a readable list of current organizations.</t>
+  </si>
+  <si>
+    <t>Given I am logged into a helper account, when I view the organizations view, I am given access to only the helper specific controls</t>
+  </si>
+  <si>
+    <t>Given I am logged into a manager account, when I view the organizations view, I am given access to only the manager specific controls</t>
+  </si>
+  <si>
+    <t>As a user, I want to view an organization’s details so I can know more about it</t>
+  </si>
+  <si>
+    <t>Given I am viewing the organizations, when I select an organization, I can see its details.</t>
+  </si>
+  <si>
+    <t>Given I am viewing an organization’s details, when I click back, the system returns me to the organization list.</t>
+  </si>
+  <si>
+    <t>As a manager, I want to edit an organization so I can update its information if it changes.</t>
+  </si>
+  <si>
+    <t>Given I am logged into a manager account, when I view an organization in the list/org detail, then I see the text field to edit it</t>
+  </si>
+  <si>
+    <t>Given I am logged into a manager account, when I click the edit button, then the edits are saved.</t>
+  </si>
+  <si>
+    <t>Given I am editing the org, when I submit the edit, then the org is edited in the system</t>
+  </si>
+  <si>
+    <t>Given I am editing the org, when I submit the edit, then the needs with the organization are updated</t>
+  </si>
+  <si>
+    <t>HS; 7/27; need does not update after org does. tends to also break some other needs and orgs related functions that are performed after it</t>
+  </si>
+  <si>
+    <t>As a manager, I want to create an organization so it can be affiliated with needs in the system.</t>
+  </si>
+  <si>
+    <t>Given I am logged into my manager account, when I view the list of organizations, I see a button to add an organization.</t>
+  </si>
+  <si>
+    <t>Given I am logged into my manager account, when I go to create an organization, the system shows me the form to do so.</t>
+  </si>
+  <si>
+    <t>Given the form has some required fields blank, when I click create, the system refuses the request and warns me of the missing data.</t>
+  </si>
+  <si>
+    <t>Given the form has all the required information and is not present in the system, when I click create, the organization is added to the system and I am routed to the organization's view.</t>
+  </si>
+  <si>
+    <t>Given the form has all the required information but is already present in the system, when I click create, the system informs me and refuses the request.</t>
+  </si>
+  <si>
+    <t>Given I am creating an organization, when I click the cancel button, the system asks me to confirm the cancellation.</t>
+  </si>
+  <si>
+    <t>Given I want to cancel creating an organization, when I click confirm, the system reroutes me to the organizations view and does not create an organization</t>
+  </si>
+  <si>
+    <t>Given I do not want to cancel creating an organization, when I click cancel on the cancel confirmation view, the system lets me continue creating an organization</t>
+  </si>
+  <si>
+    <t>Given I have created an organization, when I look at the list of organizations, then new organization is shown in its contents.</t>
+  </si>
+  <si>
+    <t>As a manager, I want to delete an organization so their affiliations can be removed from the system.</t>
+  </si>
+  <si>
+    <t>Given I am logged into my manager account, when I view an organization in the list and/or org detail view, I see a button to delete it.</t>
+  </si>
+  <si>
+    <t>Given I am logged into my manager account, when I click the delete button, i am asked to confirm org deletion.</t>
+  </si>
+  <si>
+    <t>Given I am deleting the org, when I click confirm, the org is removed from the system.</t>
+  </si>
+  <si>
+    <t>Given I am deleting the org, when I click confirm, all needs affiliated with that org are deleted.</t>
+  </si>
+  <si>
+    <t>Given I am not deleting the org, when I click cancel, the org remains in the system.</t>
+  </si>
+  <si>
+    <t>As a user, I want to be able to view proposals created by all helpers so I can see what proposals have been made.</t>
+  </si>
+  <si>
+    <t>Given I am logged into my account, I can see a link to the proposals list in the navbar</t>
+  </si>
+  <si>
+    <t>Given I am logged into my account, when I navigate to the proposals list, I can see the readable list of proposals that have been made</t>
+  </si>
+  <si>
+    <t>Given I am logged into a helper account, when I view the proposal view, I am given access to only the helper specific controls</t>
+  </si>
+  <si>
+    <t>Given I am logged into a manager account, when I view the proposal view, I am given access to only the manager specific controls</t>
+  </si>
+  <si>
+    <t>As a user, I want to view the details of a proposal so I can know more about it.</t>
+  </si>
+  <si>
+    <t>Given I am viewing the proposal, when I select a proposal, I can see its details.</t>
+  </si>
+  <si>
+    <t>Given I am viewing a proposal’s details, when I click back, the system returns me to the proposal list.</t>
+  </si>
+  <si>
+    <t>As a helper, I want to see the status of a proposal so I can know if it is unreviewed, approved, or rejected.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my account, when I am viewing the proposal list, I see a visual indicator of its status.</t>
+  </si>
+  <si>
+    <t>Given I am logged into my account, when I am viewing a proposal’s details, I see a visual indicator of its status.</t>
+  </si>
+  <si>
+    <t>As a user, I want to see votes for and against a proposal to help determine its suitability for the system.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my manager account, when I view a proposal, I can see the number of votes for and against the proposal.</t>
+  </si>
+  <si>
+    <t>As a manager, I want to add or remove an organization to a need so that I can record their affiliation with that need</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a manger, when I try to create a need, then the organization field appears in the form</t>
+  </si>
+  <si>
+    <t>Given I have added an organization, when I click the update need button, then the organization is updated and associated with that need</t>
+  </si>
+  <si>
+    <t>Given I have selected the 'No Org' option, when I click the update need button, then the need is affiliated with no organization</t>
+  </si>
+  <si>
+    <t>HS; 7/27; vestigial acceptance criteria from before we changed how our orgs and needs would interact</t>
+  </si>
+  <si>
+    <t>Given I do not want to add orgs, when I click cancel, then the  need is unchanged</t>
+  </si>
+  <si>
+    <t>Given I am using the Edit Need page, when I view the edit need's options, then I get an option to edit the organization of the need.</t>
+  </si>
+  <si>
+    <t>As a user, I want to sort/filter cupboards by organization so I can view needs by their affiliation.</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a user, when I view the cupboard, then I can also view the list of available organizations.</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a user, when I select any organizations in the cupboard's list, then I only get search results of needs affiliated with the selected organization.</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a user, when I do not select any organization in the cupboard's list, then the search for needs doesn't restrict itself to any organizations</t>
+  </si>
+  <si>
+    <t>As a helper, I want to know what needs are affiliated with each organization so that I can contribute to the desired organizations</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a user, when I view a need's details, then the need's organization should be visible</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a user, when I view a need in the cupboard, then the need's organization should be visible with the corresponding need</t>
+  </si>
+  <si>
+    <t>Given I am logged in as a user, when I click on the organization of the need, then I am taken to the details page of that organization</t>
+  </si>
+  <si>
+    <t>As a helper, I want to create need proposals so that they can be reviewed for addition to the system.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my helper account, when I click the create proposal button, the system shows me the form to create a new one.</t>
+  </si>
+  <si>
+    <t>Given the form has all the required information and is not present in the system, when I click create, the proposal is added to the system and I am routed to the proposal list view.</t>
+  </si>
+  <si>
+    <t>Given I am creating a proposal, when I click the cancel button, the system asks me to confirm the cancellation.</t>
+  </si>
+  <si>
+    <t>Given I want to cancel creating a proposal, when I click confirm, the system reroutes me to the proposal list view and does not create a proposal</t>
+  </si>
+  <si>
+    <t>Given I do not want to cancel creating a proposal, when I click cancel on the cancel confirmation view, the system lets me continue creating a proposal</t>
+  </si>
+  <si>
+    <t>Given I have created a proposal, when I look at the list of proposals, the new proposal is shown in its contents.</t>
+  </si>
+  <si>
+    <t>As a Helper, I want to be able to vote on a proposal so I can show my approval of the proposed need.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my helper account, when I view a proposal, there is a visual indication that I can vote for or against it.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my helper account, when I click vote for or vote against, the proposal's vote count updates by 1 in that direction.</t>
+  </si>
+  <si>
+    <t>Given I have already cast a vote in one direction, when I click that same direction again, my vote is removed. When I click the opposite direction instead, my vote switches to that direction.</t>
+  </si>
+  <si>
+    <t>As a user, I want to search the proposals so I can view only the ones that meet certain criteria</t>
+  </si>
+  <si>
+    <t>Given I am logged into my account, when I view the proposals, I can see a search bar.</t>
+  </si>
+  <si>
+    <t>Given I type in a string to search bar, when I click the search button, the system only displays proposals include that name.</t>
+  </si>
+  <si>
+    <t>Given the string is empty,  when I click the search button, the system shows all proposals.</t>
+  </si>
+  <si>
+    <t>As a manager, I want to approve proposals that are suitable for the system so they can be added as needs.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to a manager account, when I view a proposal, I have the option to approve it.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my manager account, when I accept a proposal, the system updates the status of the proposal to accepted.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my manager account, when I accept a proposal, the system converts it to a Need</t>
+  </si>
+  <si>
+    <t>As a manager, I want to reject proposals that are not suitable for the system so I can prevent them from being added as a need.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to a manager account, when I view a proposal, I have the option to reject it.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my manager account, when I reject a proposal, the system updates the status of the proposal to rejected.</t>
+  </si>
+  <si>
+    <t>Given I am logged in to my manager account, when I reject a proposal, Needs remain unchanged.</t>
+  </si>
 </sst>
 </file>
 
@@ -377,7 +623,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -412,6 +658,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9EAD3"/>
         <bgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E0E3"/>
+        <bgColor rgb="FFD0E0E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9DAF8"/>
+        <bgColor rgb="FFC9DAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCFE2F3"/>
+        <bgColor rgb="FFCFE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D2E9"/>
+        <bgColor rgb="FFD9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAD1DC"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -465,7 +741,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="38">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -496,11 +772,8 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -525,14 +798,53 @@
     <xf borderId="1" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="9" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="8" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3893,8 +4205,12 @@
       <c r="D2" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="13"/>
+      <c r="E2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -3917,18 +4233,22 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="14"/>
+      <c r="A3" s="13"/>
       <c r="B3" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="12"/>
-      <c r="F3" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
@@ -3951,18 +4271,22 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="14"/>
+      <c r="A4" s="13"/>
       <c r="B4" s="11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" s="12"/>
-      <c r="F4" s="13"/>
+      <c r="D4" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -3985,18 +4309,22 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="14"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="13"/>
+      <c r="D5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -4019,18 +4347,22 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="14"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
+        <v>22</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -4053,18 +4385,22 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="14"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="13"/>
+        <v>24</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -4087,18 +4423,22 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="16"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
+        <v>26</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -4122,19 +4462,23 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="12"/>
-      <c r="F9" s="13"/>
+      <c r="D9" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -4157,18 +4501,22 @@
       <c r="Z9" s="2"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="14"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E10" s="12"/>
-      <c r="F10" s="13"/>
+      <c r="D10" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -4191,18 +4539,22 @@
       <c r="Z10" s="2"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="14"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
+      <c r="D11" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -4225,18 +4577,22 @@
       <c r="Z11" s="2"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="14"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13"/>
+      <c r="D12" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -4259,18 +4615,22 @@
       <c r="Z12" s="2"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="16"/>
+      <c r="A13" s="15"/>
       <c r="B13" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="12"/>
-      <c r="F13" s="13"/>
+      <c r="D13" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -4294,10 +4654,10 @@
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>13</v>
@@ -4305,8 +4665,12 @@
       <c r="D14" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="12"/>
-      <c r="F14" s="13"/>
+      <c r="E14" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -4329,9 +4693,9 @@
       <c r="Z14" s="2"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="16"/>
+      <c r="A15" s="15"/>
       <c r="B15" s="11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>13</v>
@@ -4339,8 +4703,12 @@
       <c r="D15" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13"/>
+      <c r="E15" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -4363,20 +4731,24 @@
       <c r="Z15" s="2"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="17" t="s">
-        <v>35</v>
+      <c r="A16" s="16" t="s">
+        <v>36</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" s="12"/>
-      <c r="F16" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -4399,18 +4771,22 @@
       <c r="Z16" s="2"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="14"/>
+      <c r="A17" s="13"/>
       <c r="B17" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E17" s="12"/>
-      <c r="F17" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -4433,18 +4809,22 @@
       <c r="Z17" s="2"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="14"/>
+      <c r="A18" s="13"/>
       <c r="B18" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="13"/>
+        <v>41</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -4467,18 +4847,22 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="16"/>
+      <c r="A19" s="15"/>
       <c r="B19" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="13"/>
+        <v>43</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -4501,20 +4885,24 @@
       <c r="Z19" s="2"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="17" t="s">
-        <v>43</v>
+      <c r="A20" s="16" t="s">
+        <v>44</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="13"/>
+        <v>47</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -4537,18 +4925,22 @@
       <c r="Z20" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="16"/>
+      <c r="A21" s="15"/>
       <c r="B21" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="E21" s="12"/>
-      <c r="F21" s="13"/>
+      <c r="E21" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
@@ -4571,20 +4963,24 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="18" t="s">
-        <v>48</v>
+      <c r="A22" s="17" t="s">
+        <v>49</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="E22" s="12"/>
-      <c r="F22" s="13"/>
+        <v>51</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -4607,18 +5003,22 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="14"/>
+      <c r="A23" s="13"/>
       <c r="B23" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E23" s="12"/>
-      <c r="F23" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -4641,18 +5041,22 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="16"/>
+      <c r="A24" s="15"/>
       <c r="B24" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E24" s="12"/>
-      <c r="F24" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -4675,20 +5079,24 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="18" t="s">
-        <v>53</v>
+      <c r="A25" s="17" t="s">
+        <v>54</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="E25" s="12"/>
-      <c r="F25" s="13"/>
+        <v>51</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -4711,18 +5119,22 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="16"/>
+      <c r="A26" s="15"/>
       <c r="B26" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E26" s="12"/>
-      <c r="F26" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
@@ -4745,20 +5157,24 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="19" t="s">
-        <v>56</v>
+      <c r="A27" s="18" t="s">
+        <v>57</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
@@ -4781,20 +5197,24 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="18" t="s">
-        <v>58</v>
+      <c r="A28" s="17" t="s">
+        <v>59</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E28" s="12"/>
-      <c r="F28" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -4817,18 +5237,22 @@
       <c r="Z28" s="2"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="16"/>
+      <c r="A29" s="15"/>
       <c r="B29" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E29" s="12"/>
-      <c r="F29" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
@@ -4851,20 +5275,24 @@
       <c r="Z29" s="2"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="18" t="s">
-        <v>62</v>
+      <c r="A30" s="17" t="s">
+        <v>63</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E30" s="12"/>
-      <c r="F30" s="13"/>
+        <v>65</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
@@ -4887,18 +5315,22 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="16"/>
+      <c r="A31" s="15"/>
       <c r="B31" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E31" s="12"/>
-      <c r="F31" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -4921,20 +5353,24 @@
       <c r="Z31" s="2"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="18" t="s">
-        <v>66</v>
+      <c r="A32" s="17" t="s">
+        <v>67</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E32" s="12"/>
-      <c r="F32" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -4957,18 +5393,22 @@
       <c r="Z32" s="2"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="14"/>
+      <c r="A33" s="13"/>
       <c r="B33" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C33" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E33" s="12"/>
-      <c r="F33" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -4991,18 +5431,22 @@
       <c r="Z33" s="2"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="16"/>
+      <c r="A34" s="15"/>
       <c r="B34" s="11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C34" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E34" s="12"/>
-      <c r="F34" s="13"/>
+        <v>61</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -5025,20 +5469,24 @@
       <c r="Z34" s="2"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="20" t="s">
-        <v>70</v>
+      <c r="A35" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C35" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="13"/>
+        <v>38</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -5061,18 +5509,22 @@
       <c r="Z35" s="2"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="14"/>
+      <c r="A36" s="13"/>
       <c r="B36" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C36" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="E36" s="12"/>
-      <c r="F36" s="13"/>
+        <v>74</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -5095,18 +5547,22 @@
       <c r="Z36" s="2"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="16"/>
+      <c r="A37" s="15"/>
       <c r="B37" s="11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C37" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="E37" s="12"/>
-      <c r="F37" s="13"/>
+        <v>76</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -5129,11 +5585,11 @@
       <c r="Z37" s="2"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="20" t="s">
-        <v>76</v>
+      <c r="A38" s="19" t="s">
+        <v>77</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C38" s="10" t="s">
         <v>13</v>
@@ -5141,8 +5597,12 @@
       <c r="D38" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E38" s="12"/>
-      <c r="F38" s="13"/>
+      <c r="E38" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -5165,9 +5625,9 @@
       <c r="Z38" s="2"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="14"/>
+      <c r="A39" s="13"/>
       <c r="B39" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C39" s="10" t="s">
         <v>13</v>
@@ -5175,8 +5635,12 @@
       <c r="D39" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="12"/>
-      <c r="F39" s="13"/>
+      <c r="E39" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -5199,9 +5663,9 @@
       <c r="Z39" s="2"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="16"/>
+      <c r="A40" s="15"/>
       <c r="B40" s="11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C40" s="10" t="s">
         <v>13</v>
@@ -5209,8 +5673,12 @@
       <c r="D40" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E40" s="12"/>
-      <c r="F40" s="13"/>
+      <c r="E40" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -5233,11 +5701,11 @@
       <c r="Z40" s="2"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="20" t="s">
-        <v>80</v>
+      <c r="A41" s="19" t="s">
+        <v>81</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C41" s="10" t="s">
         <v>13</v>
@@ -5245,8 +5713,12 @@
       <c r="D41" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E41" s="12"/>
-      <c r="F41" s="13"/>
+      <c r="E41" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -5269,18 +5741,22 @@
       <c r="Z41" s="2"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="14"/>
+      <c r="A42" s="13"/>
       <c r="B42" s="11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C42" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="E42" s="12"/>
-      <c r="F42" s="13"/>
+        <v>84</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -5303,9 +5779,9 @@
       <c r="Z42" s="2"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="14"/>
+      <c r="A43" s="13"/>
       <c r="B43" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>13</v>
@@ -5313,8 +5789,12 @@
       <c r="D43" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E43" s="12"/>
-      <c r="F43" s="13"/>
+      <c r="E43" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -5337,9 +5817,9 @@
       <c r="Z43" s="2"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="16"/>
+      <c r="A44" s="15"/>
       <c r="B44" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C44" s="10" t="s">
         <v>13</v>
@@ -5347,8 +5827,12 @@
       <c r="D44" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E44" s="12"/>
-      <c r="F44" s="13"/>
+      <c r="E44" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
@@ -5371,20 +5855,24 @@
       <c r="Z44" s="2"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="21" t="s">
-        <v>86</v>
+      <c r="A45" s="20" t="s">
+        <v>87</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="E45" s="12"/>
-      <c r="F45" s="13"/>
+        <v>89</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
@@ -5407,18 +5895,22 @@
       <c r="Z45" s="2"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="16"/>
+      <c r="A46" s="15"/>
       <c r="B46" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="E46" s="12"/>
-      <c r="F46" s="13"/>
+        <v>91</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
@@ -5441,20 +5933,24 @@
       <c r="Z46" s="2"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="22" t="s">
-        <v>91</v>
+      <c r="A47" s="21" t="s">
+        <v>92</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C47" s="10" t="s">
         <v>13</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="E47" s="12"/>
-      <c r="F47" s="13"/>
+        <v>94</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
@@ -5477,12 +5973,20 @@
       <c r="Z47" s="2"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="23"/>
-      <c r="B48" s="24"/>
-      <c r="C48" s="25"/>
+      <c r="A48" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B48" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C48" s="24"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="25"/>
-      <c r="F48" s="2"/>
+      <c r="E48" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -5505,12 +6009,17 @@
       <c r="Z48" s="2"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="23"/>
-      <c r="B49" s="24"/>
-      <c r="C49" s="25"/>
+      <c r="B49" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C49" s="24"/>
       <c r="D49" s="2"/>
-      <c r="E49" s="25"/>
-      <c r="F49" s="2"/>
+      <c r="E49" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
@@ -5533,12 +6042,17 @@
       <c r="Z49" s="2"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="25"/>
+      <c r="B50" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="C50" s="24"/>
       <c r="D50" s="2"/>
-      <c r="E50" s="25"/>
-      <c r="F50" s="2"/>
+      <c r="E50" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
@@ -5561,12 +6075,17 @@
       <c r="Z50" s="2"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="25"/>
+      <c r="B51" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" s="24"/>
       <c r="D51" s="2"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="2"/>
+      <c r="E51" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
@@ -5589,12 +6108,20 @@
       <c r="Z51" s="2"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="25"/>
+      <c r="A52" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="B52" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C52" s="24"/>
       <c r="D52" s="2"/>
-      <c r="E52" s="25"/>
-      <c r="F52" s="2"/>
+      <c r="E52" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
@@ -5617,12 +6144,17 @@
       <c r="Z52" s="2"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="25"/>
+      <c r="B53" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="C53" s="24"/>
       <c r="D53" s="2"/>
-      <c r="E53" s="25"/>
-      <c r="F53" s="2"/>
+      <c r="E53" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
@@ -5645,12 +6177,20 @@
       <c r="Z53" s="2"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="25"/>
+      <c r="A54" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B54" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="C54" s="24"/>
       <c r="D54" s="2"/>
-      <c r="E54" s="25"/>
-      <c r="F54" s="2"/>
+      <c r="E54" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -5673,12 +6213,17 @@
       <c r="Z54" s="2"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="25"/>
+      <c r="B55" s="29" t="s">
+        <v>105</v>
+      </c>
+      <c r="C55" s="24"/>
       <c r="D55" s="2"/>
-      <c r="E55" s="25"/>
-      <c r="F55" s="2"/>
+      <c r="E55" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
@@ -5701,12 +6246,17 @@
       <c r="Z55" s="2"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="25"/>
+      <c r="B56" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C56" s="24"/>
       <c r="D56" s="2"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="2"/>
+      <c r="E56" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
@@ -5729,12 +6279,17 @@
       <c r="Z56" s="2"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="25"/>
+      <c r="B57" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="C57" s="24"/>
       <c r="D57" s="2"/>
-      <c r="E57" s="25"/>
-      <c r="F57" s="2"/>
+      <c r="E57" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>108</v>
+      </c>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
@@ -5757,12 +6312,20 @@
       <c r="Z57" s="2"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="25"/>
+      <c r="A58" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="B58" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="C58" s="24"/>
       <c r="D58" s="2"/>
-      <c r="E58" s="25"/>
-      <c r="F58" s="2"/>
+      <c r="E58" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
@@ -5785,12 +6348,17 @@
       <c r="Z58" s="2"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="25"/>
+      <c r="B59" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="C59" s="24"/>
       <c r="D59" s="2"/>
-      <c r="E59" s="25"/>
-      <c r="F59" s="2"/>
+      <c r="E59" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
@@ -5813,12 +6381,17 @@
       <c r="Z59" s="2"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="25"/>
+      <c r="B60" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C60" s="24"/>
       <c r="D60" s="2"/>
-      <c r="E60" s="25"/>
-      <c r="F60" s="2"/>
+      <c r="E60" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
@@ -5841,12 +6414,17 @@
       <c r="Z60" s="2"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="25"/>
+      <c r="B61" s="30" t="s">
+        <v>113</v>
+      </c>
+      <c r="C61" s="24"/>
       <c r="D61" s="2"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="2"/>
+      <c r="E61" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F61" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
@@ -5869,12 +6447,17 @@
       <c r="Z61" s="2"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="25"/>
+      <c r="B62" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="C62" s="24"/>
       <c r="D62" s="2"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="2"/>
+      <c r="E62" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
@@ -5897,12 +6480,17 @@
       <c r="Z62" s="2"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="25"/>
+      <c r="B63" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="C63" s="24"/>
       <c r="D63" s="2"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="2"/>
+      <c r="E63" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
@@ -5925,12 +6513,17 @@
       <c r="Z63" s="2"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="25"/>
+      <c r="B64" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="C64" s="24"/>
       <c r="D64" s="2"/>
-      <c r="E64" s="25"/>
-      <c r="F64" s="2"/>
+      <c r="E64" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
@@ -5953,12 +6546,17 @@
       <c r="Z64" s="2"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="25"/>
+      <c r="B65" s="30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C65" s="24"/>
       <c r="D65" s="2"/>
-      <c r="E65" s="25"/>
-      <c r="F65" s="2"/>
+      <c r="E65" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
@@ -5981,12 +6579,17 @@
       <c r="Z65" s="2"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="25"/>
+      <c r="B66" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C66" s="24"/>
       <c r="D66" s="2"/>
-      <c r="E66" s="25"/>
-      <c r="F66" s="2"/>
+      <c r="E66" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F66" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
@@ -6009,12 +6612,20 @@
       <c r="Z66" s="2"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="25"/>
+      <c r="A67" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" s="31" t="s">
+        <v>120</v>
+      </c>
+      <c r="C67" s="24"/>
       <c r="D67" s="2"/>
-      <c r="E67" s="25"/>
-      <c r="F67" s="2"/>
+      <c r="E67" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F67" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
@@ -6037,12 +6648,17 @@
       <c r="Z67" s="2"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="25"/>
+      <c r="B68" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="C68" s="24"/>
       <c r="D68" s="2"/>
-      <c r="E68" s="25"/>
-      <c r="F68" s="2"/>
+      <c r="E68" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F68" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
@@ -6065,12 +6681,17 @@
       <c r="Z68" s="2"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="25"/>
+      <c r="B69" s="31" t="s">
+        <v>122</v>
+      </c>
+      <c r="C69" s="24"/>
       <c r="D69" s="2"/>
-      <c r="E69" s="25"/>
-      <c r="F69" s="2"/>
+      <c r="E69" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F69" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
@@ -6093,12 +6714,17 @@
       <c r="Z69" s="2"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="25"/>
+      <c r="B70" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="C70" s="24"/>
       <c r="D70" s="2"/>
-      <c r="E70" s="25"/>
-      <c r="F70" s="2"/>
+      <c r="E70" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F70" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
@@ -6121,12 +6747,17 @@
       <c r="Z70" s="2"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="25"/>
+      <c r="B71" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="C71" s="24"/>
       <c r="D71" s="2"/>
-      <c r="E71" s="25"/>
-      <c r="F71" s="2"/>
+      <c r="E71" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F71" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
@@ -6149,12 +6780,20 @@
       <c r="Z71" s="2"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="2"/>
-      <c r="B72" s="2"/>
-      <c r="C72" s="25"/>
+      <c r="A72" s="32" t="s">
+        <v>125</v>
+      </c>
+      <c r="B72" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="C72" s="24"/>
       <c r="D72" s="2"/>
-      <c r="E72" s="25"/>
-      <c r="F72" s="2"/>
+      <c r="E72" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
@@ -6177,12 +6816,17 @@
       <c r="Z72" s="2"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="25"/>
+      <c r="B73" s="32" t="s">
+        <v>127</v>
+      </c>
+      <c r="C73" s="24"/>
       <c r="D73" s="2"/>
-      <c r="E73" s="25"/>
-      <c r="F73" s="2"/>
+      <c r="E73" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F73" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
@@ -6205,12 +6849,17 @@
       <c r="Z73" s="2"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
-      <c r="C74" s="25"/>
+      <c r="B74" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="C74" s="24"/>
       <c r="D74" s="2"/>
-      <c r="E74" s="25"/>
-      <c r="F74" s="2"/>
+      <c r="E74" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F74" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
@@ -6233,12 +6882,17 @@
       <c r="Z74" s="2"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="2"/>
-      <c r="B75" s="2"/>
-      <c r="C75" s="25"/>
+      <c r="B75" s="32" t="s">
+        <v>129</v>
+      </c>
+      <c r="C75" s="24"/>
       <c r="D75" s="2"/>
-      <c r="E75" s="25"/>
-      <c r="F75" s="2"/>
+      <c r="E75" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F75" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
@@ -6261,12 +6915,20 @@
       <c r="Z75" s="2"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-      <c r="C76" s="25"/>
+      <c r="A76" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="B76" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="C76" s="24"/>
       <c r="D76" s="2"/>
-      <c r="E76" s="25"/>
-      <c r="F76" s="2"/>
+      <c r="E76" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
@@ -6289,12 +6951,17 @@
       <c r="Z76" s="2"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="25"/>
+      <c r="B77" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="C77" s="24"/>
       <c r="D77" s="2"/>
-      <c r="E77" s="25"/>
-      <c r="F77" s="2"/>
+      <c r="E77" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F77" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
@@ -6317,12 +6984,20 @@
       <c r="Z77" s="2"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="25"/>
+      <c r="A78" s="34" t="s">
+        <v>133</v>
+      </c>
+      <c r="B78" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="C78" s="24"/>
       <c r="D78" s="2"/>
-      <c r="E78" s="25"/>
-      <c r="F78" s="2"/>
+      <c r="E78" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F78" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
@@ -6345,12 +7020,17 @@
       <c r="Z78" s="2"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="25"/>
+      <c r="B79" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="C79" s="24"/>
       <c r="D79" s="2"/>
-      <c r="E79" s="25"/>
-      <c r="F79" s="2"/>
+      <c r="E79" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F79" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
@@ -6373,12 +7053,20 @@
       <c r="Z79" s="2"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="25"/>
+      <c r="A80" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B80" s="35" t="s">
+        <v>137</v>
+      </c>
+      <c r="C80" s="24"/>
       <c r="D80" s="2"/>
-      <c r="E80" s="25"/>
-      <c r="F80" s="2"/>
+      <c r="E80" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F80" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
@@ -6401,12 +7089,20 @@
       <c r="Z80" s="2"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="25"/>
+      <c r="A81" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="B81" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="C81" s="24"/>
       <c r="D81" s="2"/>
-      <c r="E81" s="25"/>
-      <c r="F81" s="2"/>
+      <c r="E81" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F81" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
@@ -6429,12 +7125,17 @@
       <c r="Z81" s="2"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="25"/>
+      <c r="B82" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="C82" s="24"/>
       <c r="D82" s="2"/>
-      <c r="E82" s="25"/>
-      <c r="F82" s="2"/>
+      <c r="E82" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F82" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
@@ -6457,12 +7158,17 @@
       <c r="Z82" s="2"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
-      <c r="C83" s="25"/>
+      <c r="B83" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="C83" s="24"/>
       <c r="D83" s="2"/>
-      <c r="E83" s="25"/>
-      <c r="F83" s="2"/>
+      <c r="E83" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="F83" s="12" t="s">
+        <v>142</v>
+      </c>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
@@ -6485,12 +7191,17 @@
       <c r="Z83" s="2"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="25"/>
+      <c r="B84" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="C84" s="24"/>
       <c r="D84" s="2"/>
-      <c r="E84" s="25"/>
-      <c r="F84" s="2"/>
+      <c r="E84" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="F84" s="12" t="s">
+        <v>142</v>
+      </c>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
@@ -6513,12 +7224,17 @@
       <c r="Z84" s="2"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="25"/>
+      <c r="B85" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C85" s="24"/>
       <c r="D85" s="2"/>
-      <c r="E85" s="25"/>
-      <c r="F85" s="2"/>
+      <c r="E85" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F85" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
@@ -6541,12 +7257,20 @@
       <c r="Z85" s="2"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="25"/>
+      <c r="A86" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="B86" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="C86" s="24"/>
       <c r="D86" s="2"/>
-      <c r="E86" s="25"/>
-      <c r="F86" s="2"/>
+      <c r="E86" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
@@ -6569,12 +7293,17 @@
       <c r="Z86" s="2"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="2"/>
-      <c r="B87" s="2"/>
-      <c r="C87" s="25"/>
+      <c r="B87" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="C87" s="24"/>
       <c r="D87" s="2"/>
-      <c r="E87" s="25"/>
-      <c r="F87" s="2"/>
+      <c r="E87" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
@@ -6597,12 +7326,17 @@
       <c r="Z87" s="2"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="2"/>
-      <c r="B88" s="2"/>
-      <c r="C88" s="25"/>
+      <c r="B88" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="C88" s="24"/>
       <c r="D88" s="2"/>
-      <c r="E88" s="25"/>
-      <c r="F88" s="2"/>
+      <c r="E88" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F88" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
@@ -6625,12 +7359,20 @@
       <c r="Z88" s="2"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
-      <c r="C89" s="25"/>
+      <c r="A89" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="B89" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="C89" s="24"/>
       <c r="D89" s="2"/>
-      <c r="E89" s="25"/>
-      <c r="F89" s="2"/>
+      <c r="E89" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F89" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
@@ -6653,12 +7395,17 @@
       <c r="Z89" s="2"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="2"/>
-      <c r="B90" s="2"/>
-      <c r="C90" s="25"/>
+      <c r="B90" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="C90" s="24"/>
       <c r="D90" s="2"/>
-      <c r="E90" s="25"/>
-      <c r="F90" s="2"/>
+      <c r="E90" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F90" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
@@ -6681,12 +7428,17 @@
       <c r="Z90" s="2"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
-      <c r="C91" s="25"/>
+      <c r="B91" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="C91" s="24"/>
       <c r="D91" s="2"/>
-      <c r="E91" s="25"/>
-      <c r="F91" s="2"/>
+      <c r="E91" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F91" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
@@ -6709,12 +7461,20 @@
       <c r="Z91" s="2"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-      <c r="C92" s="25"/>
+      <c r="A92" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="B92" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="C92" s="24"/>
       <c r="D92" s="2"/>
-      <c r="E92" s="25"/>
-      <c r="F92" s="2"/>
+      <c r="E92" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F92" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
@@ -6737,12 +7497,17 @@
       <c r="Z92" s="2"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="2"/>
-      <c r="B93" s="2"/>
-      <c r="C93" s="25"/>
+      <c r="B93" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="C93" s="24"/>
       <c r="D93" s="2"/>
-      <c r="E93" s="25"/>
-      <c r="F93" s="2"/>
+      <c r="E93" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F93" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
@@ -6765,12 +7530,17 @@
       <c r="Z93" s="2"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="25"/>
+      <c r="B94" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="C94" s="24"/>
       <c r="D94" s="2"/>
-      <c r="E94" s="25"/>
-      <c r="F94" s="2"/>
+      <c r="E94" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F94" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
@@ -6793,12 +7563,17 @@
       <c r="Z94" s="2"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="2"/>
-      <c r="B95" s="2"/>
-      <c r="C95" s="25"/>
+      <c r="B95" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="C95" s="24"/>
       <c r="D95" s="2"/>
-      <c r="E95" s="25"/>
-      <c r="F95" s="2"/>
+      <c r="E95" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
@@ -6821,12 +7596,17 @@
       <c r="Z95" s="2"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="2"/>
-      <c r="B96" s="2"/>
-      <c r="C96" s="25"/>
+      <c r="B96" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="C96" s="24"/>
       <c r="D96" s="2"/>
-      <c r="E96" s="25"/>
-      <c r="F96" s="2"/>
+      <c r="E96" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F96" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
@@ -6849,12 +7629,17 @@
       <c r="Z96" s="2"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="2"/>
-      <c r="B97" s="2"/>
-      <c r="C97" s="25"/>
+      <c r="B97" s="29" t="s">
+        <v>157</v>
+      </c>
+      <c r="C97" s="24"/>
       <c r="D97" s="2"/>
-      <c r="E97" s="25"/>
-      <c r="F97" s="2"/>
+      <c r="E97" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
@@ -6877,12 +7662,17 @@
       <c r="Z97" s="2"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="2"/>
-      <c r="B98" s="2"/>
-      <c r="C98" s="25"/>
+      <c r="B98" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="C98" s="24"/>
       <c r="D98" s="2"/>
-      <c r="E98" s="25"/>
-      <c r="F98" s="2"/>
+      <c r="E98" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F98" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
@@ -6905,12 +7695,17 @@
       <c r="Z98" s="2"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="2"/>
-      <c r="B99" s="2"/>
-      <c r="C99" s="25"/>
+      <c r="B99" s="29" t="s">
+        <v>159</v>
+      </c>
+      <c r="C99" s="24"/>
       <c r="D99" s="2"/>
-      <c r="E99" s="25"/>
-      <c r="F99" s="2"/>
+      <c r="E99" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>
@@ -6933,12 +7728,20 @@
       <c r="Z99" s="2"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="2"/>
-      <c r="B100" s="2"/>
-      <c r="C100" s="25"/>
+      <c r="A100" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="B100" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="C100" s="24"/>
       <c r="D100" s="2"/>
-      <c r="E100" s="25"/>
-      <c r="F100" s="2"/>
+      <c r="E100" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F100" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
       <c r="I100" s="2"/>
@@ -6961,12 +7764,17 @@
       <c r="Z100" s="2"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="2"/>
-      <c r="B101" s="2"/>
-      <c r="C101" s="25"/>
+      <c r="B101" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="C101" s="24"/>
       <c r="D101" s="2"/>
-      <c r="E101" s="25"/>
-      <c r="F101" s="2"/>
+      <c r="E101" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F101" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
       <c r="I101" s="2"/>
@@ -6989,12 +7797,17 @@
       <c r="Z101" s="2"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="2"/>
-      <c r="B102" s="2"/>
-      <c r="C102" s="25"/>
+      <c r="B102" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="C102" s="24"/>
       <c r="D102" s="2"/>
-      <c r="E102" s="25"/>
-      <c r="F102" s="2"/>
+      <c r="E102" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F102" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
       <c r="I102" s="2"/>
@@ -7017,12 +7830,20 @@
       <c r="Z102" s="2"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="2"/>
-      <c r="B103" s="2"/>
-      <c r="C103" s="25"/>
+      <c r="A103" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="B103" s="31" t="s">
+        <v>165</v>
+      </c>
+      <c r="C103" s="24"/>
       <c r="D103" s="2"/>
-      <c r="E103" s="25"/>
-      <c r="F103" s="2"/>
+      <c r="E103" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F103" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
@@ -7045,12 +7866,17 @@
       <c r="Z103" s="2"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="2"/>
-      <c r="B104" s="2"/>
-      <c r="C104" s="25"/>
+      <c r="B104" s="31" t="s">
+        <v>166</v>
+      </c>
+      <c r="C104" s="24"/>
       <c r="D104" s="2"/>
-      <c r="E104" s="25"/>
-      <c r="F104" s="2"/>
+      <c r="E104" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F104" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
@@ -7073,12 +7899,17 @@
       <c r="Z104" s="2"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="2"/>
-      <c r="B105" s="2"/>
-      <c r="C105" s="25"/>
+      <c r="B105" s="31" t="s">
+        <v>167</v>
+      </c>
+      <c r="C105" s="24"/>
       <c r="D105" s="2"/>
-      <c r="E105" s="25"/>
-      <c r="F105" s="2"/>
+      <c r="E105" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F105" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
       <c r="I105" s="2"/>
@@ -7101,12 +7932,20 @@
       <c r="Z105" s="2"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="2"/>
-      <c r="B106" s="2"/>
-      <c r="C106" s="25"/>
+      <c r="A106" s="32" t="s">
+        <v>168</v>
+      </c>
+      <c r="B106" s="32" t="s">
+        <v>169</v>
+      </c>
+      <c r="C106" s="24"/>
       <c r="D106" s="2"/>
-      <c r="E106" s="25"/>
-      <c r="F106" s="2"/>
+      <c r="E106" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F106" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
@@ -7129,12 +7968,17 @@
       <c r="Z106" s="2"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="2"/>
-      <c r="B107" s="2"/>
-      <c r="C107" s="25"/>
+      <c r="B107" s="32" t="s">
+        <v>170</v>
+      </c>
+      <c r="C107" s="24"/>
       <c r="D107" s="2"/>
-      <c r="E107" s="25"/>
-      <c r="F107" s="2"/>
+      <c r="E107" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F107" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
@@ -7157,12 +8001,17 @@
       <c r="Z107" s="2"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="2"/>
-      <c r="B108" s="2"/>
-      <c r="C108" s="25"/>
+      <c r="B108" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="C108" s="24"/>
       <c r="D108" s="2"/>
-      <c r="E108" s="25"/>
-      <c r="F108" s="2"/>
+      <c r="E108" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F108" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
       <c r="I108" s="2"/>
@@ -7185,12 +8034,20 @@
       <c r="Z108" s="2"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="A109" s="2"/>
-      <c r="B109" s="2"/>
-      <c r="C109" s="25"/>
+      <c r="A109" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="B109" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="C109" s="24"/>
       <c r="D109" s="2"/>
-      <c r="E109" s="25"/>
-      <c r="F109" s="2"/>
+      <c r="E109" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F109" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
       <c r="I109" s="2"/>
@@ -7213,12 +8070,17 @@
       <c r="Z109" s="2"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="2"/>
-      <c r="B110" s="2"/>
-      <c r="C110" s="25"/>
+      <c r="B110" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="C110" s="24"/>
       <c r="D110" s="2"/>
-      <c r="E110" s="25"/>
-      <c r="F110" s="2"/>
+      <c r="E110" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F110" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
       <c r="I110" s="2"/>
@@ -7241,12 +8103,17 @@
       <c r="Z110" s="2"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="A111" s="2"/>
-      <c r="B111" s="2"/>
-      <c r="C111" s="25"/>
+      <c r="B111" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="C111" s="24"/>
       <c r="D111" s="2"/>
-      <c r="E111" s="25"/>
-      <c r="F111" s="2"/>
+      <c r="E111" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F111" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
       <c r="I111" s="2"/>
@@ -7269,11 +8136,11 @@
       <c r="Z111" s="2"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="A112" s="2"/>
-      <c r="B112" s="2"/>
-      <c r="C112" s="25"/>
+      <c r="A112" s="12"/>
+      <c r="B112" s="12"/>
+      <c r="C112" s="24"/>
       <c r="D112" s="2"/>
-      <c r="E112" s="25"/>
+      <c r="E112" s="24"/>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
@@ -7297,11 +8164,11 @@
       <c r="Z112" s="2"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="A113" s="2"/>
-      <c r="B113" s="2"/>
-      <c r="C113" s="25"/>
+      <c r="A113" s="12"/>
+      <c r="B113" s="12"/>
+      <c r="C113" s="24"/>
       <c r="D113" s="2"/>
-      <c r="E113" s="25"/>
+      <c r="E113" s="24"/>
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
@@ -7325,11 +8192,11 @@
       <c r="Z113" s="2"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="A114" s="2"/>
-      <c r="B114" s="2"/>
-      <c r="C114" s="25"/>
+      <c r="A114" s="12"/>
+      <c r="B114" s="12"/>
+      <c r="C114" s="24"/>
       <c r="D114" s="2"/>
-      <c r="E114" s="25"/>
+      <c r="E114" s="24"/>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
@@ -7353,11 +8220,11 @@
       <c r="Z114" s="2"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="A115" s="2"/>
-      <c r="B115" s="2"/>
-      <c r="C115" s="25"/>
+      <c r="A115" s="12"/>
+      <c r="B115" s="12"/>
+      <c r="C115" s="24"/>
       <c r="D115" s="2"/>
-      <c r="E115" s="25"/>
+      <c r="E115" s="24"/>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
@@ -7381,11 +8248,11 @@
       <c r="Z115" s="2"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="2"/>
-      <c r="B116" s="2"/>
-      <c r="C116" s="25"/>
+      <c r="A116" s="12"/>
+      <c r="B116" s="12"/>
+      <c r="C116" s="24"/>
       <c r="D116" s="2"/>
-      <c r="E116" s="25"/>
+      <c r="E116" s="24"/>
       <c r="F116" s="2"/>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
@@ -7409,11 +8276,11 @@
       <c r="Z116" s="2"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="A117" s="2"/>
-      <c r="B117" s="2"/>
-      <c r="C117" s="25"/>
+      <c r="A117" s="12"/>
+      <c r="B117" s="12"/>
+      <c r="C117" s="24"/>
       <c r="D117" s="2"/>
-      <c r="E117" s="25"/>
+      <c r="E117" s="24"/>
       <c r="F117" s="2"/>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
@@ -7437,11 +8304,11 @@
       <c r="Z117" s="2"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
-      <c r="A118" s="2"/>
-      <c r="B118" s="2"/>
-      <c r="C118" s="25"/>
+      <c r="A118" s="12"/>
+      <c r="B118" s="12"/>
+      <c r="C118" s="24"/>
       <c r="D118" s="2"/>
-      <c r="E118" s="25"/>
+      <c r="E118" s="24"/>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
@@ -7465,11 +8332,11 @@
       <c r="Z118" s="2"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="A119" s="2"/>
-      <c r="B119" s="2"/>
-      <c r="C119" s="25"/>
+      <c r="A119" s="12"/>
+      <c r="B119" s="12"/>
+      <c r="C119" s="24"/>
       <c r="D119" s="2"/>
-      <c r="E119" s="25"/>
+      <c r="E119" s="24"/>
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
@@ -7493,11 +8360,11 @@
       <c r="Z119" s="2"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="A120" s="2"/>
-      <c r="B120" s="2"/>
-      <c r="C120" s="25"/>
+      <c r="A120" s="12"/>
+      <c r="B120" s="12"/>
+      <c r="C120" s="24"/>
       <c r="D120" s="2"/>
-      <c r="E120" s="25"/>
+      <c r="E120" s="24"/>
       <c r="F120" s="2"/>
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
@@ -7521,11 +8388,11 @@
       <c r="Z120" s="2"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="A121" s="2"/>
-      <c r="B121" s="2"/>
-      <c r="C121" s="25"/>
+      <c r="A121" s="12"/>
+      <c r="B121" s="12"/>
+      <c r="C121" s="24"/>
       <c r="D121" s="2"/>
-      <c r="E121" s="25"/>
+      <c r="E121" s="24"/>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
@@ -7551,9 +8418,9 @@
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
-      <c r="C122" s="25"/>
+      <c r="C122" s="24"/>
       <c r="D122" s="2"/>
-      <c r="E122" s="25"/>
+      <c r="E122" s="24"/>
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
@@ -7579,9 +8446,9 @@
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
-      <c r="C123" s="25"/>
+      <c r="C123" s="24"/>
       <c r="D123" s="2"/>
-      <c r="E123" s="25"/>
+      <c r="E123" s="24"/>
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
@@ -7607,9 +8474,9 @@
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
-      <c r="C124" s="25"/>
+      <c r="C124" s="24"/>
       <c r="D124" s="2"/>
-      <c r="E124" s="25"/>
+      <c r="E124" s="24"/>
       <c r="F124" s="2"/>
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
@@ -7635,9 +8502,9 @@
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
-      <c r="C125" s="25"/>
+      <c r="C125" s="24"/>
       <c r="D125" s="2"/>
-      <c r="E125" s="25"/>
+      <c r="E125" s="24"/>
       <c r="F125" s="2"/>
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
@@ -7663,9 +8530,9 @@
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
-      <c r="C126" s="25"/>
+      <c r="C126" s="24"/>
       <c r="D126" s="2"/>
-      <c r="E126" s="25"/>
+      <c r="E126" s="24"/>
       <c r="F126" s="2"/>
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
@@ -7691,9 +8558,9 @@
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
-      <c r="C127" s="25"/>
+      <c r="C127" s="24"/>
       <c r="D127" s="2"/>
-      <c r="E127" s="25"/>
+      <c r="E127" s="24"/>
       <c r="F127" s="2"/>
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
@@ -7719,9 +8586,9 @@
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
-      <c r="C128" s="25"/>
+      <c r="C128" s="24"/>
       <c r="D128" s="2"/>
-      <c r="E128" s="25"/>
+      <c r="E128" s="24"/>
       <c r="F128" s="2"/>
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
@@ -7747,9 +8614,9 @@
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
-      <c r="C129" s="25"/>
+      <c r="C129" s="24"/>
       <c r="D129" s="2"/>
-      <c r="E129" s="25"/>
+      <c r="E129" s="24"/>
       <c r="F129" s="2"/>
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
@@ -7775,9 +8642,9 @@
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
-      <c r="C130" s="25"/>
+      <c r="C130" s="24"/>
       <c r="D130" s="2"/>
-      <c r="E130" s="25"/>
+      <c r="E130" s="24"/>
       <c r="F130" s="2"/>
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
@@ -7803,9 +8670,9 @@
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
-      <c r="C131" s="25"/>
+      <c r="C131" s="24"/>
       <c r="D131" s="2"/>
-      <c r="E131" s="25"/>
+      <c r="E131" s="24"/>
       <c r="F131" s="2"/>
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
@@ -7831,9 +8698,9 @@
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
-      <c r="C132" s="25"/>
+      <c r="C132" s="24"/>
       <c r="D132" s="2"/>
-      <c r="E132" s="25"/>
+      <c r="E132" s="24"/>
       <c r="F132" s="2"/>
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
@@ -7859,9 +8726,9 @@
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
-      <c r="C133" s="25"/>
+      <c r="C133" s="24"/>
       <c r="D133" s="2"/>
-      <c r="E133" s="25"/>
+      <c r="E133" s="24"/>
       <c r="F133" s="2"/>
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
@@ -7887,9 +8754,9 @@
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
-      <c r="C134" s="25"/>
+      <c r="C134" s="24"/>
       <c r="D134" s="2"/>
-      <c r="E134" s="25"/>
+      <c r="E134" s="24"/>
       <c r="F134" s="2"/>
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
@@ -7915,9 +8782,9 @@
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
-      <c r="C135" s="25"/>
+      <c r="C135" s="24"/>
       <c r="D135" s="2"/>
-      <c r="E135" s="25"/>
+      <c r="E135" s="24"/>
       <c r="F135" s="2"/>
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
@@ -7943,9 +8810,9 @@
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
-      <c r="C136" s="25"/>
+      <c r="C136" s="24"/>
       <c r="D136" s="2"/>
-      <c r="E136" s="25"/>
+      <c r="E136" s="24"/>
       <c r="F136" s="2"/>
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
@@ -7971,9 +8838,9 @@
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
-      <c r="C137" s="25"/>
+      <c r="C137" s="24"/>
       <c r="D137" s="2"/>
-      <c r="E137" s="25"/>
+      <c r="E137" s="24"/>
       <c r="F137" s="2"/>
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
@@ -7999,9 +8866,9 @@
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
-      <c r="C138" s="25"/>
+      <c r="C138" s="24"/>
       <c r="D138" s="2"/>
-      <c r="E138" s="25"/>
+      <c r="E138" s="24"/>
       <c r="F138" s="2"/>
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
@@ -8027,9 +8894,9 @@
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
-      <c r="C139" s="25"/>
+      <c r="C139" s="24"/>
       <c r="D139" s="2"/>
-      <c r="E139" s="25"/>
+      <c r="E139" s="24"/>
       <c r="F139" s="2"/>
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
@@ -8055,9 +8922,9 @@
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
-      <c r="C140" s="25"/>
+      <c r="C140" s="24"/>
       <c r="D140" s="2"/>
-      <c r="E140" s="25"/>
+      <c r="E140" s="24"/>
       <c r="F140" s="2"/>
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
@@ -8083,9 +8950,9 @@
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
-      <c r="C141" s="25"/>
+      <c r="C141" s="24"/>
       <c r="D141" s="2"/>
-      <c r="E141" s="25"/>
+      <c r="E141" s="24"/>
       <c r="F141" s="2"/>
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
@@ -8111,9 +8978,9 @@
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
-      <c r="C142" s="25"/>
+      <c r="C142" s="24"/>
       <c r="D142" s="2"/>
-      <c r="E142" s="25"/>
+      <c r="E142" s="24"/>
       <c r="F142" s="2"/>
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
@@ -8139,9 +9006,9 @@
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
-      <c r="C143" s="25"/>
+      <c r="C143" s="24"/>
       <c r="D143" s="2"/>
-      <c r="E143" s="25"/>
+      <c r="E143" s="24"/>
       <c r="F143" s="2"/>
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
@@ -8167,9 +9034,9 @@
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
-      <c r="C144" s="25"/>
+      <c r="C144" s="24"/>
       <c r="D144" s="2"/>
-      <c r="E144" s="25"/>
+      <c r="E144" s="24"/>
       <c r="F144" s="2"/>
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
@@ -8195,9 +9062,9 @@
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
-      <c r="C145" s="25"/>
+      <c r="C145" s="24"/>
       <c r="D145" s="2"/>
-      <c r="E145" s="25"/>
+      <c r="E145" s="24"/>
       <c r="F145" s="2"/>
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
@@ -8223,9 +9090,9 @@
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
-      <c r="C146" s="25"/>
+      <c r="C146" s="24"/>
       <c r="D146" s="2"/>
-      <c r="E146" s="25"/>
+      <c r="E146" s="24"/>
       <c r="F146" s="2"/>
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
@@ -8251,9 +9118,9 @@
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
-      <c r="C147" s="25"/>
+      <c r="C147" s="24"/>
       <c r="D147" s="2"/>
-      <c r="E147" s="25"/>
+      <c r="E147" s="24"/>
       <c r="F147" s="2"/>
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
@@ -8279,9 +9146,9 @@
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
-      <c r="C148" s="25"/>
+      <c r="C148" s="24"/>
       <c r="D148" s="2"/>
-      <c r="E148" s="25"/>
+      <c r="E148" s="24"/>
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
@@ -8307,9 +9174,9 @@
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
-      <c r="C149" s="25"/>
+      <c r="C149" s="24"/>
       <c r="D149" s="2"/>
-      <c r="E149" s="25"/>
+      <c r="E149" s="24"/>
       <c r="F149" s="2"/>
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
@@ -8335,9 +9202,9 @@
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
-      <c r="C150" s="25"/>
+      <c r="C150" s="24"/>
       <c r="D150" s="2"/>
-      <c r="E150" s="25"/>
+      <c r="E150" s="24"/>
       <c r="F150" s="2"/>
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
@@ -8363,9 +9230,9 @@
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
-      <c r="C151" s="25"/>
+      <c r="C151" s="24"/>
       <c r="D151" s="2"/>
-      <c r="E151" s="25"/>
+      <c r="E151" s="24"/>
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
@@ -8391,9 +9258,9 @@
     <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
-      <c r="C152" s="25"/>
+      <c r="C152" s="24"/>
       <c r="D152" s="2"/>
-      <c r="E152" s="25"/>
+      <c r="E152" s="24"/>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
@@ -8419,9 +9286,9 @@
     <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
-      <c r="C153" s="25"/>
+      <c r="C153" s="24"/>
       <c r="D153" s="2"/>
-      <c r="E153" s="25"/>
+      <c r="E153" s="24"/>
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
@@ -8447,9 +9314,9 @@
     <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
-      <c r="C154" s="25"/>
+      <c r="C154" s="24"/>
       <c r="D154" s="2"/>
-      <c r="E154" s="25"/>
+      <c r="E154" s="24"/>
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
@@ -8475,9 +9342,9 @@
     <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
-      <c r="C155" s="25"/>
+      <c r="C155" s="24"/>
       <c r="D155" s="2"/>
-      <c r="E155" s="25"/>
+      <c r="E155" s="24"/>
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
@@ -8503,9 +9370,9 @@
     <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
-      <c r="C156" s="25"/>
+      <c r="C156" s="24"/>
       <c r="D156" s="2"/>
-      <c r="E156" s="25"/>
+      <c r="E156" s="24"/>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
@@ -8531,9 +9398,9 @@
     <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
-      <c r="C157" s="25"/>
+      <c r="C157" s="24"/>
       <c r="D157" s="2"/>
-      <c r="E157" s="25"/>
+      <c r="E157" s="24"/>
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
@@ -8559,9 +9426,9 @@
     <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
-      <c r="C158" s="25"/>
+      <c r="C158" s="24"/>
       <c r="D158" s="2"/>
-      <c r="E158" s="25"/>
+      <c r="E158" s="24"/>
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
@@ -8587,9 +9454,9 @@
     <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
-      <c r="C159" s="25"/>
+      <c r="C159" s="24"/>
       <c r="D159" s="2"/>
-      <c r="E159" s="25"/>
+      <c r="E159" s="24"/>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
@@ -8615,9 +9482,9 @@
     <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
-      <c r="C160" s="25"/>
+      <c r="C160" s="24"/>
       <c r="D160" s="2"/>
-      <c r="E160" s="25"/>
+      <c r="E160" s="24"/>
       <c r="F160" s="2"/>
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
@@ -8643,9 +9510,9 @@
     <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
-      <c r="C161" s="25"/>
+      <c r="C161" s="24"/>
       <c r="D161" s="2"/>
-      <c r="E161" s="25"/>
+      <c r="E161" s="24"/>
       <c r="F161" s="2"/>
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
@@ -8671,9 +9538,9 @@
     <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
-      <c r="C162" s="25"/>
+      <c r="C162" s="24"/>
       <c r="D162" s="2"/>
-      <c r="E162" s="25"/>
+      <c r="E162" s="24"/>
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
@@ -8699,9 +9566,9 @@
     <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
-      <c r="C163" s="25"/>
+      <c r="C163" s="24"/>
       <c r="D163" s="2"/>
-      <c r="E163" s="25"/>
+      <c r="E163" s="24"/>
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
@@ -8727,9 +9594,9 @@
     <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
-      <c r="C164" s="25"/>
+      <c r="C164" s="24"/>
       <c r="D164" s="2"/>
-      <c r="E164" s="25"/>
+      <c r="E164" s="24"/>
       <c r="F164" s="2"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
@@ -8755,9 +9622,9 @@
     <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
-      <c r="C165" s="25"/>
+      <c r="C165" s="24"/>
       <c r="D165" s="2"/>
-      <c r="E165" s="25"/>
+      <c r="E165" s="24"/>
       <c r="F165" s="2"/>
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
@@ -8783,9 +9650,9 @@
     <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
-      <c r="C166" s="25"/>
+      <c r="C166" s="24"/>
       <c r="D166" s="2"/>
-      <c r="E166" s="25"/>
+      <c r="E166" s="24"/>
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
@@ -8811,9 +9678,9 @@
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
-      <c r="C167" s="25"/>
+      <c r="C167" s="24"/>
       <c r="D167" s="2"/>
-      <c r="E167" s="25"/>
+      <c r="E167" s="24"/>
       <c r="F167" s="2"/>
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
@@ -8839,9 +9706,9 @@
     <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
-      <c r="C168" s="25"/>
+      <c r="C168" s="24"/>
       <c r="D168" s="2"/>
-      <c r="E168" s="25"/>
+      <c r="E168" s="24"/>
       <c r="F168" s="2"/>
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
@@ -8867,9 +9734,9 @@
     <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
-      <c r="C169" s="25"/>
+      <c r="C169" s="24"/>
       <c r="D169" s="2"/>
-      <c r="E169" s="25"/>
+      <c r="E169" s="24"/>
       <c r="F169" s="2"/>
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
@@ -8895,9 +9762,9 @@
     <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
-      <c r="C170" s="25"/>
+      <c r="C170" s="24"/>
       <c r="D170" s="2"/>
-      <c r="E170" s="25"/>
+      <c r="E170" s="24"/>
       <c r="F170" s="2"/>
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
@@ -8923,9 +9790,9 @@
     <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
-      <c r="C171" s="25"/>
+      <c r="C171" s="24"/>
       <c r="D171" s="2"/>
-      <c r="E171" s="25"/>
+      <c r="E171" s="24"/>
       <c r="F171" s="2"/>
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
@@ -8951,9 +9818,9 @@
     <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
-      <c r="C172" s="25"/>
+      <c r="C172" s="24"/>
       <c r="D172" s="2"/>
-      <c r="E172" s="25"/>
+      <c r="E172" s="24"/>
       <c r="F172" s="2"/>
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
@@ -8979,9 +9846,9 @@
     <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
-      <c r="C173" s="25"/>
+      <c r="C173" s="24"/>
       <c r="D173" s="2"/>
-      <c r="E173" s="25"/>
+      <c r="E173" s="24"/>
       <c r="F173" s="2"/>
       <c r="G173" s="2"/>
       <c r="H173" s="2"/>
@@ -9007,9 +9874,9 @@
     <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
-      <c r="C174" s="25"/>
+      <c r="C174" s="24"/>
       <c r="D174" s="2"/>
-      <c r="E174" s="25"/>
+      <c r="E174" s="24"/>
       <c r="F174" s="2"/>
       <c r="G174" s="2"/>
       <c r="H174" s="2"/>
@@ -9035,9 +9902,9 @@
     <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
-      <c r="C175" s="25"/>
+      <c r="C175" s="24"/>
       <c r="D175" s="2"/>
-      <c r="E175" s="25"/>
+      <c r="E175" s="24"/>
       <c r="F175" s="2"/>
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
@@ -9063,9 +9930,9 @@
     <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
-      <c r="C176" s="25"/>
+      <c r="C176" s="24"/>
       <c r="D176" s="2"/>
-      <c r="E176" s="25"/>
+      <c r="E176" s="24"/>
       <c r="F176" s="2"/>
       <c r="G176" s="2"/>
       <c r="H176" s="2"/>
@@ -9091,9 +9958,9 @@
     <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
-      <c r="C177" s="25"/>
+      <c r="C177" s="24"/>
       <c r="D177" s="2"/>
-      <c r="E177" s="25"/>
+      <c r="E177" s="24"/>
       <c r="F177" s="2"/>
       <c r="G177" s="2"/>
       <c r="H177" s="2"/>
@@ -9119,9 +9986,9 @@
     <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
-      <c r="C178" s="25"/>
+      <c r="C178" s="24"/>
       <c r="D178" s="2"/>
-      <c r="E178" s="25"/>
+      <c r="E178" s="24"/>
       <c r="F178" s="2"/>
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
@@ -9147,9 +10014,9 @@
     <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
-      <c r="C179" s="25"/>
+      <c r="C179" s="24"/>
       <c r="D179" s="2"/>
-      <c r="E179" s="25"/>
+      <c r="E179" s="24"/>
       <c r="F179" s="2"/>
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
@@ -9175,9 +10042,9 @@
     <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
-      <c r="C180" s="25"/>
+      <c r="C180" s="24"/>
       <c r="D180" s="2"/>
-      <c r="E180" s="25"/>
+      <c r="E180" s="24"/>
       <c r="F180" s="2"/>
       <c r="G180" s="2"/>
       <c r="H180" s="2"/>
@@ -9203,9 +10070,9 @@
     <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
-      <c r="C181" s="25"/>
+      <c r="C181" s="24"/>
       <c r="D181" s="2"/>
-      <c r="E181" s="25"/>
+      <c r="E181" s="24"/>
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
@@ -9231,9 +10098,9 @@
     <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
-      <c r="C182" s="25"/>
+      <c r="C182" s="24"/>
       <c r="D182" s="2"/>
-      <c r="E182" s="25"/>
+      <c r="E182" s="24"/>
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
@@ -9259,9 +10126,9 @@
     <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
-      <c r="C183" s="25"/>
+      <c r="C183" s="24"/>
       <c r="D183" s="2"/>
-      <c r="E183" s="25"/>
+      <c r="E183" s="24"/>
       <c r="F183" s="2"/>
       <c r="G183" s="2"/>
       <c r="H183" s="2"/>
@@ -9287,9 +10154,9 @@
     <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
-      <c r="C184" s="25"/>
+      <c r="C184" s="24"/>
       <c r="D184" s="2"/>
-      <c r="E184" s="25"/>
+      <c r="E184" s="24"/>
       <c r="F184" s="2"/>
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
@@ -9315,9 +10182,9 @@
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
-      <c r="C185" s="25"/>
+      <c r="C185" s="24"/>
       <c r="D185" s="2"/>
-      <c r="E185" s="25"/>
+      <c r="E185" s="24"/>
       <c r="F185" s="2"/>
       <c r="G185" s="2"/>
       <c r="H185" s="2"/>
@@ -9343,9 +10210,9 @@
     <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
-      <c r="C186" s="25"/>
+      <c r="C186" s="24"/>
       <c r="D186" s="2"/>
-      <c r="E186" s="25"/>
+      <c r="E186" s="24"/>
       <c r="F186" s="2"/>
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
@@ -9371,9 +10238,9 @@
     <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
-      <c r="C187" s="25"/>
+      <c r="C187" s="24"/>
       <c r="D187" s="2"/>
-      <c r="E187" s="25"/>
+      <c r="E187" s="24"/>
       <c r="F187" s="2"/>
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
@@ -9399,9 +10266,9 @@
     <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
-      <c r="C188" s="25"/>
+      <c r="C188" s="24"/>
       <c r="D188" s="2"/>
-      <c r="E188" s="25"/>
+      <c r="E188" s="24"/>
       <c r="F188" s="2"/>
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
@@ -9427,9 +10294,9 @@
     <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
-      <c r="C189" s="25"/>
+      <c r="C189" s="24"/>
       <c r="D189" s="2"/>
-      <c r="E189" s="25"/>
+      <c r="E189" s="24"/>
       <c r="F189" s="2"/>
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
@@ -9455,9 +10322,9 @@
     <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
-      <c r="C190" s="25"/>
+      <c r="C190" s="24"/>
       <c r="D190" s="2"/>
-      <c r="E190" s="25"/>
+      <c r="E190" s="24"/>
       <c r="F190" s="2"/>
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
@@ -9483,9 +10350,9 @@
     <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
-      <c r="C191" s="25"/>
+      <c r="C191" s="24"/>
       <c r="D191" s="2"/>
-      <c r="E191" s="25"/>
+      <c r="E191" s="24"/>
       <c r="F191" s="2"/>
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
@@ -9511,9 +10378,9 @@
     <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="2"/>
       <c r="B192" s="2"/>
-      <c r="C192" s="25"/>
+      <c r="C192" s="24"/>
       <c r="D192" s="2"/>
-      <c r="E192" s="25"/>
+      <c r="E192" s="24"/>
       <c r="F192" s="2"/>
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
@@ -9539,9 +10406,9 @@
     <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
-      <c r="C193" s="25"/>
+      <c r="C193" s="24"/>
       <c r="D193" s="2"/>
-      <c r="E193" s="25"/>
+      <c r="E193" s="24"/>
       <c r="F193" s="2"/>
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
@@ -9567,9 +10434,9 @@
     <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="2"/>
       <c r="B194" s="2"/>
-      <c r="C194" s="25"/>
+      <c r="C194" s="24"/>
       <c r="D194" s="2"/>
-      <c r="E194" s="25"/>
+      <c r="E194" s="24"/>
       <c r="F194" s="2"/>
       <c r="G194" s="2"/>
       <c r="H194" s="2"/>
@@ -9595,9 +10462,9 @@
     <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="2"/>
       <c r="B195" s="2"/>
-      <c r="C195" s="25"/>
+      <c r="C195" s="24"/>
       <c r="D195" s="2"/>
-      <c r="E195" s="25"/>
+      <c r="E195" s="24"/>
       <c r="F195" s="2"/>
       <c r="G195" s="2"/>
       <c r="H195" s="2"/>
@@ -9623,9 +10490,9 @@
     <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
-      <c r="C196" s="25"/>
+      <c r="C196" s="24"/>
       <c r="D196" s="2"/>
-      <c r="E196" s="25"/>
+      <c r="E196" s="24"/>
       <c r="F196" s="2"/>
       <c r="G196" s="2"/>
       <c r="H196" s="2"/>
@@ -9651,9 +10518,9 @@
     <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="2"/>
       <c r="B197" s="2"/>
-      <c r="C197" s="25"/>
+      <c r="C197" s="24"/>
       <c r="D197" s="2"/>
-      <c r="E197" s="25"/>
+      <c r="E197" s="24"/>
       <c r="F197" s="2"/>
       <c r="G197" s="2"/>
       <c r="H197" s="2"/>
@@ -9679,9 +10546,9 @@
     <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
-      <c r="C198" s="25"/>
+      <c r="C198" s="24"/>
       <c r="D198" s="2"/>
-      <c r="E198" s="25"/>
+      <c r="E198" s="24"/>
       <c r="F198" s="2"/>
       <c r="G198" s="2"/>
       <c r="H198" s="2"/>
@@ -9707,9 +10574,9 @@
     <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="2"/>
       <c r="B199" s="2"/>
-      <c r="C199" s="25"/>
+      <c r="C199" s="24"/>
       <c r="D199" s="2"/>
-      <c r="E199" s="25"/>
+      <c r="E199" s="24"/>
       <c r="F199" s="2"/>
       <c r="G199" s="2"/>
       <c r="H199" s="2"/>
@@ -9735,9 +10602,9 @@
     <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
-      <c r="C200" s="25"/>
+      <c r="C200" s="24"/>
       <c r="D200" s="2"/>
-      <c r="E200" s="25"/>
+      <c r="E200" s="24"/>
       <c r="F200" s="2"/>
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
@@ -9763,9 +10630,9 @@
     <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="2"/>
       <c r="B201" s="2"/>
-      <c r="C201" s="25"/>
+      <c r="C201" s="24"/>
       <c r="D201" s="2"/>
-      <c r="E201" s="25"/>
+      <c r="E201" s="24"/>
       <c r="F201" s="2"/>
       <c r="G201" s="2"/>
       <c r="H201" s="2"/>
@@ -9791,9 +10658,9 @@
     <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="2"/>
       <c r="B202" s="2"/>
-      <c r="C202" s="25"/>
+      <c r="C202" s="24"/>
       <c r="D202" s="2"/>
-      <c r="E202" s="25"/>
+      <c r="E202" s="24"/>
       <c r="F202" s="2"/>
       <c r="G202" s="2"/>
       <c r="H202" s="2"/>
@@ -9819,9 +10686,9 @@
     <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="2"/>
       <c r="B203" s="2"/>
-      <c r="C203" s="25"/>
+      <c r="C203" s="24"/>
       <c r="D203" s="2"/>
-      <c r="E203" s="25"/>
+      <c r="E203" s="24"/>
       <c r="F203" s="2"/>
       <c r="G203" s="2"/>
       <c r="H203" s="2"/>
@@ -9847,9 +10714,9 @@
     <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="2"/>
       <c r="B204" s="2"/>
-      <c r="C204" s="25"/>
+      <c r="C204" s="24"/>
       <c r="D204" s="2"/>
-      <c r="E204" s="25"/>
+      <c r="E204" s="24"/>
       <c r="F204" s="2"/>
       <c r="G204" s="2"/>
       <c r="H204" s="2"/>
@@ -9875,9 +10742,9 @@
     <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="2"/>
       <c r="B205" s="2"/>
-      <c r="C205" s="25"/>
+      <c r="C205" s="24"/>
       <c r="D205" s="2"/>
-      <c r="E205" s="25"/>
+      <c r="E205" s="24"/>
       <c r="F205" s="2"/>
       <c r="G205" s="2"/>
       <c r="H205" s="2"/>
@@ -9903,9 +10770,9 @@
     <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="2"/>
       <c r="B206" s="2"/>
-      <c r="C206" s="25"/>
+      <c r="C206" s="24"/>
       <c r="D206" s="2"/>
-      <c r="E206" s="25"/>
+      <c r="E206" s="24"/>
       <c r="F206" s="2"/>
       <c r="G206" s="2"/>
       <c r="H206" s="2"/>
@@ -9931,9 +10798,9 @@
     <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="2"/>
       <c r="B207" s="2"/>
-      <c r="C207" s="25"/>
+      <c r="C207" s="24"/>
       <c r="D207" s="2"/>
-      <c r="E207" s="25"/>
+      <c r="E207" s="24"/>
       <c r="F207" s="2"/>
       <c r="G207" s="2"/>
       <c r="H207" s="2"/>
@@ -9959,9 +10826,9 @@
     <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="2"/>
       <c r="B208" s="2"/>
-      <c r="C208" s="25"/>
+      <c r="C208" s="24"/>
       <c r="D208" s="2"/>
-      <c r="E208" s="25"/>
+      <c r="E208" s="24"/>
       <c r="F208" s="2"/>
       <c r="G208" s="2"/>
       <c r="H208" s="2"/>
@@ -9987,9 +10854,9 @@
     <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="2"/>
       <c r="B209" s="2"/>
-      <c r="C209" s="25"/>
+      <c r="C209" s="24"/>
       <c r="D209" s="2"/>
-      <c r="E209" s="25"/>
+      <c r="E209" s="24"/>
       <c r="F209" s="2"/>
       <c r="G209" s="2"/>
       <c r="H209" s="2"/>
@@ -10015,9 +10882,9 @@
     <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="2"/>
       <c r="B210" s="2"/>
-      <c r="C210" s="25"/>
+      <c r="C210" s="24"/>
       <c r="D210" s="2"/>
-      <c r="E210" s="25"/>
+      <c r="E210" s="24"/>
       <c r="F210" s="2"/>
       <c r="G210" s="2"/>
       <c r="H210" s="2"/>
@@ -10043,9 +10910,9 @@
     <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="2"/>
       <c r="B211" s="2"/>
-      <c r="C211" s="25"/>
+      <c r="C211" s="24"/>
       <c r="D211" s="2"/>
-      <c r="E211" s="25"/>
+      <c r="E211" s="24"/>
       <c r="F211" s="2"/>
       <c r="G211" s="2"/>
       <c r="H211" s="2"/>
@@ -10071,9 +10938,9 @@
     <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="2"/>
       <c r="B212" s="2"/>
-      <c r="C212" s="25"/>
+      <c r="C212" s="24"/>
       <c r="D212" s="2"/>
-      <c r="E212" s="25"/>
+      <c r="E212" s="24"/>
       <c r="F212" s="2"/>
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
@@ -10099,9 +10966,9 @@
     <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="2"/>
       <c r="B213" s="2"/>
-      <c r="C213" s="25"/>
+      <c r="C213" s="24"/>
       <c r="D213" s="2"/>
-      <c r="E213" s="25"/>
+      <c r="E213" s="24"/>
       <c r="F213" s="2"/>
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
@@ -10127,9 +10994,9 @@
     <row r="214" ht="15.75" customHeight="1">
       <c r="A214" s="2"/>
       <c r="B214" s="2"/>
-      <c r="C214" s="25"/>
+      <c r="C214" s="24"/>
       <c r="D214" s="2"/>
-      <c r="E214" s="25"/>
+      <c r="E214" s="24"/>
       <c r="F214" s="2"/>
       <c r="G214" s="2"/>
       <c r="H214" s="2"/>
@@ -10155,9 +11022,9 @@
     <row r="215" ht="15.75" customHeight="1">
       <c r="A215" s="2"/>
       <c r="B215" s="2"/>
-      <c r="C215" s="25"/>
+      <c r="C215" s="24"/>
       <c r="D215" s="2"/>
-      <c r="E215" s="25"/>
+      <c r="E215" s="24"/>
       <c r="F215" s="2"/>
       <c r="G215" s="2"/>
       <c r="H215" s="2"/>
@@ -10183,9 +11050,9 @@
     <row r="216" ht="15.75" customHeight="1">
       <c r="A216" s="2"/>
       <c r="B216" s="2"/>
-      <c r="C216" s="25"/>
+      <c r="C216" s="24"/>
       <c r="D216" s="2"/>
-      <c r="E216" s="25"/>
+      <c r="E216" s="24"/>
       <c r="F216" s="2"/>
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
@@ -10211,9 +11078,9 @@
     <row r="217" ht="15.75" customHeight="1">
       <c r="A217" s="2"/>
       <c r="B217" s="2"/>
-      <c r="C217" s="25"/>
+      <c r="C217" s="24"/>
       <c r="D217" s="2"/>
-      <c r="E217" s="25"/>
+      <c r="E217" s="24"/>
       <c r="F217" s="2"/>
       <c r="G217" s="2"/>
       <c r="H217" s="2"/>
@@ -10239,9 +11106,9 @@
     <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="2"/>
       <c r="B218" s="2"/>
-      <c r="C218" s="25"/>
+      <c r="C218" s="24"/>
       <c r="D218" s="2"/>
-      <c r="E218" s="25"/>
+      <c r="E218" s="24"/>
       <c r="F218" s="2"/>
       <c r="G218" s="2"/>
       <c r="H218" s="2"/>
@@ -10267,9 +11134,9 @@
     <row r="219" ht="15.75" customHeight="1">
       <c r="A219" s="2"/>
       <c r="B219" s="2"/>
-      <c r="C219" s="25"/>
+      <c r="C219" s="24"/>
       <c r="D219" s="2"/>
-      <c r="E219" s="25"/>
+      <c r="E219" s="24"/>
       <c r="F219" s="2"/>
       <c r="G219" s="2"/>
       <c r="H219" s="2"/>
@@ -10295,9 +11162,9 @@
     <row r="220" ht="15.75" customHeight="1">
       <c r="A220" s="2"/>
       <c r="B220" s="2"/>
-      <c r="C220" s="25"/>
+      <c r="C220" s="24"/>
       <c r="D220" s="2"/>
-      <c r="E220" s="25"/>
+      <c r="E220" s="24"/>
       <c r="F220" s="2"/>
       <c r="G220" s="2"/>
       <c r="H220" s="2"/>
@@ -32161,7 +33028,14 @@
       <c r="Z1000" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="30">
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="A32:A34"/>
@@ -32169,13 +33043,22 @@
     <mergeCell ref="A38:A40"/>
     <mergeCell ref="A41:A44"/>
     <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A2:A8"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A48:A51"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="A58:A66"/>
+    <mergeCell ref="A67:A71"/>
+    <mergeCell ref="A72:A75"/>
+    <mergeCell ref="A76:A77"/>
+    <mergeCell ref="A106:A108"/>
+    <mergeCell ref="A109:A111"/>
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="A86:A88"/>
+    <mergeCell ref="A89:A91"/>
+    <mergeCell ref="A92:A99"/>
+    <mergeCell ref="A100:A102"/>
+    <mergeCell ref="A103:A105"/>
   </mergeCells>
   <conditionalFormatting sqref="C2:C1000 E2:E1000">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">

</xml_diff>